<commit_message>
#47 PCB Completed Deliverables and BOM Generated
</commit_message>
<xml_diff>
--- a/Design Files/Powermodule-v9.0.0/BOM/Client_BOM.xlsx
+++ b/Design Files/Powermodule-v9.0.0/BOM/Client_BOM.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="350">
   <si>
     <t>#</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t xml:space="preserve"> Remarks</t>
+    <t>#Column Name Error:' Remarks</t>
   </si>
   <si>
     <t>Capacitor</t>
@@ -80,7 +80,7 @@
     <t>47uF</t>
   </si>
   <si>
-    <t>C2, C3, C4, C34, C56, C59, C61</t>
+    <t>C2, C3, C4, C13, C34, C56, C59, C61</t>
   </si>
   <si>
     <t>CAP CER 10UF 25V X5R 0603</t>
@@ -98,7 +98,7 @@
     <t>10uF</t>
   </si>
   <si>
-    <t>C5, C10, C12, C18, C19, C20, C21, C22, C23, C24, C25, C26, C33, C39, C40, C41, C42, C58, C62</t>
+    <t>C5, C10, C12, C14, C18, C19, C20, C21, C22, C23, C24, C25, C26, C33, C39, C40, C41, C42, C58, C62</t>
   </si>
   <si>
     <t>CAP CER 0.1UF 50V X7R 0402</t>
@@ -257,7 +257,7 @@
     <t>Diode</t>
   </si>
   <si>
-    <t>D2, D3, D4, D5, D6, D7, D8, D10, D11</t>
+    <t>D2, D3, D4, D5, D6, D7, D8, D10</t>
   </si>
   <si>
     <t>75V 200mW Single 1.25V@150mA 4ns 150mA SOD-323 Switching Diode ROHS</t>
@@ -329,12 +329,15 @@
     <t>Connectors</t>
   </si>
   <si>
-    <t>J1</t>
+    <t>J1, J11</t>
   </si>
   <si>
     <t>CONN HEADER SMD R/A 8POS 1.25MM</t>
   </si>
   <si>
+    <t>Custom</t>
+  </si>
+  <si>
     <t>SM08B-GHS-TB(LF)(SN)</t>
   </si>
   <si>
@@ -410,15 +413,6 @@
     <t>MYOUNG</t>
   </si>
   <si>
-    <t>J11</t>
-  </si>
-  <si>
-    <t>CONN HEADER SMD R/A 7POS 1.25MM</t>
-  </si>
-  <si>
-    <t>SM07B-GHS-TB(LF)(SN)</t>
-  </si>
-  <si>
     <t>Headers</t>
   </si>
   <si>
@@ -440,9 +434,6 @@
     <t>4A 2.2uH ±20% 32mΩ SMD,5.4x5.2x2mm Power Inductors ROHS</t>
   </si>
   <si>
-    <t>YSPI0520-2R2M_</t>
-  </si>
-  <si>
     <t>YSPI0520-2R2M</t>
   </si>
   <si>
@@ -491,10 +482,13 @@
     <t>NCD0603R3</t>
   </si>
   <si>
+    <t>DNP</t>
+  </si>
+  <si>
     <t>TEST POINT</t>
   </si>
   <si>
-    <t>P2, P3, P6, P7, P9, P10, P11, P12, P15, P16, P17, P18, P19, P20, P21, P22, P24, P25, P26, P27, P28, P29, P30, P31, P33, P34, P35, P36, P37, P38, P39, P43, P44, P45</t>
+    <t>P2, P3, P7, P9, P10, P11, P12, P15, P16, P17, P18, P19, P20, P21, P22, P24, P25, P26, P27, P28, P29, P30, P31, P33, P34, P35, P36, P37, P38, P39, P43, P44, P45</t>
   </si>
   <si>
     <t>Test Point ON</t>
@@ -503,10 +497,55 @@
     <t>Test-point</t>
   </si>
   <si>
+    <t>MOSFET</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>null 3A 400mW 112mΩ@4.5V,2.8A 1V@250uA P Channel SOT-23 MOSFETs ROHS</t>
+  </si>
+  <si>
+    <t>SOT-23</t>
+  </si>
+  <si>
+    <t>SI2301CDS</t>
+  </si>
+  <si>
+    <t>FUXINSEMI</t>
+  </si>
+  <si>
+    <t>Transistor</t>
+  </si>
+  <si>
+    <t>Q3, Q4</t>
+  </si>
+  <si>
+    <t>45V 300mW 100@100mA,1V 500mA NPN SOT-23 Bipolar Transistors - BJT ROHS</t>
+  </si>
+  <si>
+    <t>BC817 6B 160-400</t>
+  </si>
+  <si>
+    <t>DOWO</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>MOSFET N-CH 60V 320MA SOT23-3</t>
+  </si>
+  <si>
+    <t>2N7002KT1G</t>
+  </si>
+  <si>
+    <t>ON Semiconductor</t>
+  </si>
+  <si>
     <t>MOSFETs</t>
   </si>
   <si>
-    <t>Q1, Q7</t>
+    <t>Q7</t>
   </si>
   <si>
     <t>MOSFET P-CH 20V 6.9A 6TSOP</t>
@@ -521,51 +560,6 @@
     <t>Infineon</t>
   </si>
   <si>
-    <t>SOT-23</t>
-  </si>
-  <si>
-    <t>Q2</t>
-  </si>
-  <si>
-    <t>null 3A 400mW 112mΩ@4.5V,2.8A 1V@250uA P Channel SOT-23 MOSFETs ROHS</t>
-  </si>
-  <si>
-    <t>SI2301CDS</t>
-  </si>
-  <si>
-    <t>FUXINSEMI</t>
-  </si>
-  <si>
-    <t>Transistor</t>
-  </si>
-  <si>
-    <t>Q3, Q4</t>
-  </si>
-  <si>
-    <t>45V 300mW 100@100mA,1V 500mA NPN SOT-23 Bipolar Transistors - BJT ROHS</t>
-  </si>
-  <si>
-    <t>BC817 6B 160-400</t>
-  </si>
-  <si>
-    <t>DOWO</t>
-  </si>
-  <si>
-    <t>MOSFET</t>
-  </si>
-  <si>
-    <t>Q5, Q6</t>
-  </si>
-  <si>
-    <t>MOSFET N-CH 60V 320MA SOT23-3</t>
-  </si>
-  <si>
-    <t>2N7002KT1G</t>
-  </si>
-  <si>
-    <t>ON Semiconductor</t>
-  </si>
-  <si>
     <t>Mosfet</t>
   </si>
   <si>
@@ -581,76 +575,106 @@
     <t>SI2302CDS</t>
   </si>
   <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>RES 560 OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>Res-0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-07560RL</t>
+  </si>
+  <si>
+    <t>560R</t>
+  </si>
+  <si>
+    <t>R2, R8, R11, R12, R13, R30, R34, R59, R71, R72, R73</t>
+  </si>
+  <si>
+    <t>RES 100K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-07100KL</t>
+  </si>
+  <si>
+    <t>100K</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>RES 33.2K OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>Res-0603</t>
+  </si>
+  <si>
+    <t>RC0603FR-0733K2L</t>
+  </si>
+  <si>
+    <t>33.2K</t>
+  </si>
+  <si>
+    <t>R4, R16, R17</t>
+  </si>
+  <si>
+    <t>RES 200 OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-07200RL</t>
+  </si>
+  <si>
+    <t>200R</t>
+  </si>
+  <si>
+    <t>R5, R6, R21, R25, R26, R37, R53, R54, R61, R65, R66, R69, R70</t>
+  </si>
+  <si>
+    <t>RES 10K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-0710KL</t>
+  </si>
+  <si>
+    <t>10K</t>
+  </si>
+  <si>
+    <t>R5 is DNP</t>
+  </si>
+  <si>
     <t>Resistors</t>
   </si>
   <si>
-    <t>R1, R7</t>
+    <t>R7</t>
   </si>
   <si>
     <t>RES SMD 390 OHM 0.1% 1/16W 0402</t>
   </si>
   <si>
-    <t>Res-0402</t>
-  </si>
-  <si>
     <t>RT0402BRD07390RL</t>
   </si>
   <si>
-    <t>390R</t>
-  </si>
-  <si>
-    <t>Resistor</t>
-  </si>
-  <si>
-    <t>R2, R8, R11, R12, R13, R30, R32, R33, R34, R35, R38, R48, R59, R71, R72, R73</t>
-  </si>
-  <si>
-    <t>RES 100K OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
-    <t>RC0402FR-07100KL</t>
-  </si>
-  <si>
-    <t>100K</t>
-  </si>
-  <si>
-    <t>R3</t>
-  </si>
-  <si>
-    <t>RES 33.2K OHM 1% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>Res-0603</t>
-  </si>
-  <si>
-    <t>RC0603FR-0733K2L</t>
-  </si>
-  <si>
-    <t>33.2K</t>
-  </si>
-  <si>
-    <t>R4, R16, R17</t>
-  </si>
-  <si>
-    <t>RES 200 OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
-    <t>RC0402FR-07200RL</t>
-  </si>
-  <si>
-    <t>200R</t>
-  </si>
-  <si>
-    <t>R5, R6, R9, R10, R21, R25, R26, R37, R43, R53, R54, R61, R65, R66, R69, R70</t>
-  </si>
-  <si>
-    <t>RES 10K OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
-    <t>RC0402FR-0710KL</t>
-  </si>
-  <si>
-    <t>10K</t>
+    <t>R9, R19, R22, R31, R32, R33</t>
+  </si>
+  <si>
+    <t>RES SMD 1K OHM 1% 1/5W 0402</t>
+  </si>
+  <si>
+    <t>CRCW04021K00FKEDHP</t>
+  </si>
+  <si>
+    <t>Vishay Dale</t>
+  </si>
+  <si>
+    <t>1K</t>
+  </si>
+  <si>
+    <t>R10, R43, R60</t>
   </si>
   <si>
     <t>R14, R15, R29, R57</t>
@@ -680,27 +704,9 @@
     <t>27R</t>
   </si>
   <si>
-    <t>R19, R22, R31, R44</t>
-  </si>
-  <si>
-    <t>RES SMD 1K OHM 1% 1/5W 0402</t>
-  </si>
-  <si>
-    <t>CRCW04021K00FKEDHP</t>
-  </si>
-  <si>
-    <t>Vishay Dale</t>
-  </si>
-  <si>
-    <t>1K</t>
-  </si>
-  <si>
     <t>R23, R24</t>
   </si>
   <si>
-    <t>DNP</t>
-  </si>
-  <si>
     <t>R27, R28</t>
   </si>
   <si>
@@ -722,6 +728,9 @@
     <t>20K</t>
   </si>
   <si>
+    <t>R44</t>
+  </si>
+  <si>
     <t>R45</t>
   </si>
   <si>
@@ -746,18 +755,6 @@
     <t>200K</t>
   </si>
   <si>
-    <t>R47</t>
-  </si>
-  <si>
-    <t>RES SMD 97.6KOHM 0.1% 1/16W 0402</t>
-  </si>
-  <si>
-    <t>RT0402BRD0797K6L</t>
-  </si>
-  <si>
-    <t>97.6K</t>
-  </si>
-  <si>
     <t>R51</t>
   </si>
   <si>
@@ -806,9 +803,6 @@
     <t>0R</t>
   </si>
   <si>
-    <t>R60</t>
-  </si>
-  <si>
     <t>R62</t>
   </si>
   <si>
@@ -869,10 +863,7 @@
     <t>Panasonic</t>
   </si>
   <si>
-    <t>SW2</t>
-  </si>
-  <si>
-    <t>SW3</t>
+    <t>SW2, SW3</t>
   </si>
   <si>
     <t>Switch Tactile N.O. SPST Round Button Gull Wing 0.05A 12VDC 100000Cycles 1.57N SMD</t>
@@ -902,19 +893,16 @@
     <t>Texas Instruments</t>
   </si>
   <si>
-    <t>Opam</t>
-  </si>
-  <si>
     <t>U2</t>
   </si>
   <si>
-    <t>IC CMOS 1 CIRCUIT SOT23-5</t>
+    <t>IC BUF NON-INVERT 5.5V SOT23-5</t>
   </si>
   <si>
     <t>SOT-23-5</t>
   </si>
   <si>
-    <t>TLV271IDBVR</t>
+    <t>SN74LV1T34DBVR</t>
   </si>
   <si>
     <t>U3</t>
@@ -1101,10 +1089,18 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1140,6 +1136,22 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="10"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1726,189 +1738,194 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2236,11 +2253,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K78"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="1" customWidth="1"/>
+    <col min="2" max="2" width="3.14285714285714" style="2" customWidth="1"/>
+    <col min="3" max="3" width="18.7142857142857" style="2" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="26.5714285714286" customWidth="1"/>
@@ -2252,90 +2269,92 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" spans="1:11">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
+      <c r="A1" s="3"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" ht="15.75" spans="1:11">
-      <c r="A2" s="2"/>
-      <c r="B2" s="5" t="s">
+      <c r="A2" s="3"/>
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" ht="36.75" spans="1:11">
-      <c r="A3" s="2"/>
-      <c r="B3" s="7">
+      <c r="A3" s="3"/>
+      <c r="B3" s="8">
         <f>ROW(B3)-ROW($B$2)</f>
         <v>1</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="10">
         <v>4</v>
       </c>
-      <c r="K3" s="9"/>
+      <c r="K3" s="10"/>
     </row>
     <row r="4" ht="15.75" spans="1:11">
-      <c r="A4" s="2"/>
-      <c r="B4" s="7">
+      <c r="A4" s="3"/>
+      <c r="B4" s="8">
         <f>ROW(B4)-ROW($B$2)</f>
         <v>2</v>
       </c>
-      <c r="C4" s="11"/>
+      <c r="C4" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="D4" s="12" t="s">
         <v>17</v>
       </c>
@@ -2355,49 +2374,49 @@
         <v>22</v>
       </c>
       <c r="J4" s="12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K4" s="12"/>
     </row>
     <row r="5" ht="24.75" spans="1:11">
-      <c r="A5" s="2"/>
-      <c r="B5" s="7">
+      <c r="A5" s="3"/>
+      <c r="B5" s="8">
         <f>ROW(B5)-ROW($B$2)</f>
         <v>3</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="9">
-        <v>19</v>
-      </c>
-      <c r="K5" s="9"/>
+      <c r="J5" s="10">
+        <v>20</v>
+      </c>
+      <c r="K5" s="10"/>
     </row>
     <row r="6" ht="15.75" spans="1:11">
-      <c r="A6" s="2"/>
-      <c r="B6" s="7">
+      <c r="A6" s="3"/>
+      <c r="B6" s="8">
         <f>ROW(B6)-ROW($B$2)</f>
         <v>4</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="12" t="s">
@@ -2424,44 +2443,44 @@
       <c r="K6" s="12"/>
     </row>
     <row r="7" ht="15.75" spans="1:11">
-      <c r="A7" s="2"/>
-      <c r="B7" s="7">
+      <c r="A7" s="3"/>
+      <c r="B7" s="8">
         <f>ROW(B7)-ROW($B$2)</f>
         <v>5</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="10">
         <v>6</v>
       </c>
-      <c r="K7" s="9"/>
+      <c r="K7" s="10"/>
     </row>
     <row r="8" ht="36.75" spans="1:11">
-      <c r="A8" s="2"/>
-      <c r="B8" s="7">
+      <c r="A8" s="3"/>
+      <c r="B8" s="8">
         <f>ROW(B8)-ROW($B$2)</f>
         <v>6</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="14" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="12" t="s">
@@ -2488,44 +2507,44 @@
       <c r="K8" s="12"/>
     </row>
     <row r="9" ht="15.75" spans="1:11">
-      <c r="A9" s="2"/>
-      <c r="B9" s="7">
+      <c r="A9" s="3"/>
+      <c r="B9" s="8">
         <f>ROW(B9)-ROW($B$2)</f>
         <v>7</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="10">
         <v>2</v>
       </c>
-      <c r="K9" s="9"/>
+      <c r="K9" s="10"/>
     </row>
     <row r="10" ht="15.75" spans="1:11">
-      <c r="A10" s="2"/>
-      <c r="B10" s="7">
+      <c r="A10" s="3"/>
+      <c r="B10" s="8">
         <f>ROW(B10)-ROW($B$2)</f>
         <v>8</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="14" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="12" t="s">
@@ -2552,44 +2571,44 @@
       <c r="K10" s="12"/>
     </row>
     <row r="11" ht="15.75" spans="1:11">
-      <c r="A11" s="2"/>
-      <c r="B11" s="7">
+      <c r="A11" s="3"/>
+      <c r="B11" s="8">
         <f>ROW(B11)-ROW($B$2)</f>
         <v>9</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="10">
         <v>1</v>
       </c>
-      <c r="K11" s="9"/>
+      <c r="K11" s="10"/>
     </row>
     <row r="12" ht="36.75" spans="1:11">
-      <c r="A12" s="2"/>
-      <c r="B12" s="7">
+      <c r="A12" s="3"/>
+      <c r="B12" s="8">
         <f>ROW(B12)-ROW($B$2)</f>
         <v>10</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="14" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="12" t="s">
@@ -2616,44 +2635,44 @@
       <c r="K12" s="12"/>
     </row>
     <row r="13" ht="15.75" spans="1:11">
-      <c r="A13" s="2"/>
-      <c r="B13" s="7">
+      <c r="A13" s="3"/>
+      <c r="B13" s="8">
         <f>ROW(B13)-ROW($B$2)</f>
         <v>11</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G13" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="10">
         <v>2</v>
       </c>
-      <c r="K13" s="9"/>
+      <c r="K13" s="10"/>
     </row>
     <row r="14" ht="24.75" spans="1:11">
-      <c r="A14" s="2"/>
-      <c r="B14" s="7">
+      <c r="A14" s="3"/>
+      <c r="B14" s="8">
         <f>ROW(B14)-ROW($B$2)</f>
         <v>12</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="14" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="12" t="s">
@@ -2680,44 +2699,44 @@
       <c r="K14" s="12"/>
     </row>
     <row r="15" ht="15.75" spans="1:11">
-      <c r="A15" s="2"/>
-      <c r="B15" s="7">
+      <c r="A15" s="3"/>
+      <c r="B15" s="8">
         <f>ROW(B15)-ROW($B$2)</f>
         <v>13</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="G15" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="I15" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="J15" s="9">
+      <c r="J15" s="10">
         <v>1</v>
       </c>
-      <c r="K15" s="9"/>
+      <c r="K15" s="10"/>
     </row>
     <row r="16" ht="24.75" spans="1:11">
-      <c r="A16" s="2"/>
-      <c r="B16" s="7">
+      <c r="A16" s="3"/>
+      <c r="B16" s="8">
         <f>ROW(B16)-ROW($B$2)</f>
         <v>14</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="14" t="s">
         <v>75</v>
       </c>
       <c r="D16" s="12" t="s">
@@ -2739,49 +2758,49 @@
         <v>81</v>
       </c>
       <c r="J16" s="12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K16" s="12"/>
     </row>
     <row r="17" ht="24.75" spans="1:11">
-      <c r="A17" s="2"/>
-      <c r="B17" s="7">
+      <c r="A17" s="3"/>
+      <c r="B17" s="8">
         <f>ROW(B17)-ROW($B$2)</f>
         <v>15</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="G17" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="I17" s="13" t="s">
+      <c r="I17" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="10">
         <v>2</v>
       </c>
-      <c r="K17" s="9"/>
+      <c r="K17" s="10"/>
     </row>
     <row r="18" ht="24.75" spans="1:11">
-      <c r="A18" s="2"/>
-      <c r="B18" s="7">
+      <c r="A18" s="3"/>
+      <c r="B18" s="8">
         <f>ROW(B18)-ROW($B$2)</f>
         <v>16</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="14" t="s">
         <v>87</v>
       </c>
       <c r="D18" s="12" t="s">
@@ -2807,45 +2826,45 @@
       </c>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" ht="15.75" spans="1:11">
-      <c r="A19" s="2"/>
-      <c r="B19" s="7">
+    <row r="19" spans="1:11">
+      <c r="A19" s="3"/>
+      <c r="B19" s="8">
         <f>ROW(B19)-ROW($B$2)</f>
         <v>17</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="G19" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="I19" s="13" t="s">
+      <c r="I19" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J19" s="9">
+      <c r="J19" s="10">
         <v>1</v>
       </c>
-      <c r="K19" s="9"/>
-    </row>
-    <row r="20" ht="15.75" spans="1:11">
-      <c r="A20" s="2"/>
-      <c r="B20" s="7">
+      <c r="K19" s="10"/>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="3"/>
+      <c r="B20" s="8">
         <f>ROW(B20)-ROW($B$2)</f>
         <v>18</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="14" t="s">
         <v>99</v>
       </c>
       <c r="D20" s="12" t="s">
@@ -2858,72 +2877,74 @@
         <v>102</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I20" s="13" t="s">
         <v>81</v>
       </c>
       <c r="J20" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="12"/>
     </row>
-    <row r="21" ht="15.75" spans="1:11">
-      <c r="A21" s="2"/>
-      <c r="B21" s="7">
+    <row r="21" spans="1:11">
+      <c r="A21" s="3"/>
+      <c r="B21" s="8">
         <f>ROW(B21)-ROW($B$2)</f>
         <v>19</v>
       </c>
-      <c r="C21" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="C21" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="D21" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="E21" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="G21" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="H21" s="9" t="s">
+      <c r="F21" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G21" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="I21" s="13" t="s">
+      <c r="H21" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I21" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J21" s="9">
+      <c r="J21" s="10">
         <v>1</v>
       </c>
-      <c r="K21" s="9"/>
+      <c r="K21" s="10"/>
     </row>
     <row r="22" ht="15.75" spans="1:11">
-      <c r="A22" s="2"/>
-      <c r="B22" s="7">
+      <c r="A22" s="3"/>
+      <c r="B22" s="8">
         <f>ROW(B22)-ROW($B$2)</f>
         <v>20</v>
       </c>
-      <c r="C22" s="11"/>
+      <c r="C22" s="9" t="s">
+        <v>105</v>
+      </c>
       <c r="D22" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="H22" s="12" t="s">
         <v>109</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="F22" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="G22" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>108</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>81</v>
@@ -2934,60 +2955,60 @@
       <c r="K22" s="12"/>
     </row>
     <row r="23" ht="24.75" spans="1:11">
-      <c r="A23" s="2"/>
-      <c r="B23" s="7">
+      <c r="A23" s="3"/>
+      <c r="B23" s="8">
         <f>ROW(B23)-ROW($B$2)</f>
         <v>21</v>
       </c>
-      <c r="C23" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="C23" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="D23" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="F23" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="G23" s="10" t="s">
+      <c r="E23" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="H23" s="9" t="s">
+      <c r="F23" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G23" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="I23" s="13" t="s">
+      <c r="H23" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="I23" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J23" s="9">
+      <c r="J23" s="10">
         <v>4</v>
       </c>
-      <c r="K23" s="9"/>
-    </row>
-    <row r="24" ht="15.75" spans="1:11">
-      <c r="A24" s="2"/>
-      <c r="B24" s="7">
+      <c r="K23" s="10"/>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="3"/>
+      <c r="B24" s="8">
         <f>ROW(B24)-ROW($B$2)</f>
         <v>22</v>
       </c>
-      <c r="C24" s="11" t="s">
-        <v>117</v>
+      <c r="C24" s="14" t="s">
+        <v>118</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I24" s="13" t="s">
         <v>81</v>
@@ -2998,60 +3019,60 @@
       <c r="K24" s="12"/>
     </row>
     <row r="25" ht="36.75" spans="1:11">
-      <c r="A25" s="2"/>
-      <c r="B25" s="7">
+      <c r="A25" s="3"/>
+      <c r="B25" s="8">
         <f>ROW(B25)-ROW($B$2)</f>
         <v>23</v>
       </c>
-      <c r="C25" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="D25" s="9" t="s">
+      <c r="C25" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="D25" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="E25" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="G25" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="H25" s="9" t="s">
+      <c r="F25" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G25" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="I25" s="13" t="s">
+      <c r="H25" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I25" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J25" s="9">
+      <c r="J25" s="10">
         <v>1</v>
       </c>
-      <c r="K25" s="9"/>
-    </row>
-    <row r="26" ht="15.75" spans="1:11">
-      <c r="A26" s="2"/>
-      <c r="B26" s="7">
+      <c r="K25" s="10"/>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="3"/>
+      <c r="B26" s="8">
         <f>ROW(B26)-ROW($B$2)</f>
         <v>24</v>
       </c>
-      <c r="C26" s="11" t="s">
-        <v>99</v>
+      <c r="C26" s="14" t="s">
+        <v>128</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>129</v>
+        <v>102</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I26" s="13" t="s">
         <v>81</v>
@@ -3061,251 +3082,251 @@
       </c>
       <c r="K26" s="12"/>
     </row>
-    <row r="27" ht="15.75" spans="1:11">
-      <c r="A27" s="2"/>
-      <c r="B27" s="7">
+    <row r="27" ht="24.75" spans="1:11">
+      <c r="A27" s="3"/>
+      <c r="B27" s="8">
         <f>ROW(B27)-ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="E27" s="10" t="s">
+      <c r="C27" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="D27" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="G27" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="I27" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="J27" s="9">
+      <c r="E27" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="I27" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="J27" s="10">
         <v>1</v>
       </c>
-      <c r="K27" s="9"/>
-    </row>
-    <row r="28" ht="24.75" spans="1:11">
-      <c r="A28" s="2"/>
-      <c r="B28" s="7">
+      <c r="K27" s="10"/>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="3"/>
+      <c r="B28" s="8">
         <f>ROW(B28)-ROW($B$2)</f>
         <v>26</v>
       </c>
-      <c r="C28" s="11" t="s">
-        <v>134</v>
-      </c>
+      <c r="C28" s="14"/>
       <c r="D28" s="12" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>137</v>
+        <v>102</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>139</v>
+        <v>27</v>
       </c>
       <c r="I28" s="13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J28" s="12">
         <v>1</v>
       </c>
       <c r="K28" s="12"/>
     </row>
-    <row r="29" ht="15.75" spans="1:11">
-      <c r="A29" s="2"/>
-      <c r="B29" s="7">
+    <row r="29" ht="24.75" spans="1:11">
+      <c r="A29" s="3"/>
+      <c r="B29" s="8">
         <f>ROW(B29)-ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="E29" s="10" t="s">
+      <c r="C29" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="D29" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="G29" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="I29" s="10" t="s">
+      <c r="E29" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="J29" s="9">
-        <v>1</v>
-      </c>
-      <c r="K29" s="9"/>
+      <c r="F29" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="H29" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="J29" s="10">
+        <v>3</v>
+      </c>
+      <c r="K29" s="10"/>
     </row>
     <row r="30" ht="24.75" spans="1:11">
-      <c r="A30" s="2"/>
-      <c r="B30" s="7">
+      <c r="A30" s="3"/>
+      <c r="B30" s="8">
         <f>ROW(B30)-ROW($B$2)</f>
         <v>28</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="F30" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="D30" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="E30" s="13" t="s">
+      <c r="G30" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="H30" s="12" t="s">
         <v>147</v>
-      </c>
-      <c r="F30" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="G30" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="H30" s="12" t="s">
-        <v>150</v>
       </c>
       <c r="I30" s="13" t="s">
         <v>81</v>
       </c>
       <c r="J30" s="12">
-        <v>3</v>
-      </c>
-      <c r="K30" s="12"/>
-    </row>
-    <row r="31" ht="24.75" spans="1:11">
-      <c r="A31" s="2"/>
-      <c r="B31" s="7">
+        <v>1</v>
+      </c>
+      <c r="K30" s="21" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="31" s="1" customFormat="1" ht="48.75" spans="1:11">
+      <c r="A31" s="15"/>
+      <c r="B31" s="16">
         <f>ROW(B31)-ROW($B$2)</f>
         <v>29</v>
       </c>
-      <c r="C31" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="E31" s="10" t="s">
+      <c r="C31" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="F31" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="G31" s="10" t="s">
+      <c r="D31" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="H31" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="I31" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="J31" s="9">
-        <v>1</v>
-      </c>
-      <c r="K31" s="9"/>
-    </row>
-    <row r="32" ht="48.75" spans="1:11">
-      <c r="A32" s="2"/>
-      <c r="B32" s="7">
+      <c r="E31" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="H31" s="18"/>
+      <c r="I31" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="J31" s="18">
+        <v>33</v>
+      </c>
+      <c r="K31" s="18"/>
+    </row>
+    <row r="32" ht="36.75" spans="1:11">
+      <c r="A32" s="3"/>
+      <c r="B32" s="8">
         <f>ROW(B32)-ROW($B$2)</f>
         <v>30</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="E32" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="F32" s="15" t="s">
+      <c r="D32" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="G32" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="H32" s="15"/>
-      <c r="I32" s="16" t="s">
+      <c r="E32" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G32" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="H32" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="I32" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="J32" s="15">
-        <v>34</v>
-      </c>
-      <c r="K32" s="15"/>
-    </row>
-    <row r="33" spans="1:11">
-      <c r="A33" s="2"/>
-      <c r="B33" s="7">
+      <c r="J32" s="12">
+        <v>1</v>
+      </c>
+      <c r="K32" s="12"/>
+    </row>
+    <row r="33" ht="36.75" spans="1:11">
+      <c r="A33" s="3"/>
+      <c r="B33" s="8">
         <f>ROW(B33)-ROW($B$2)</f>
         <v>31</v>
       </c>
-      <c r="C33" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="D33" s="9" t="s">
+      <c r="C33" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="F33" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="E33" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="F33" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="G33" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="I33" s="13" t="s">
+      <c r="G33" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="I33" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J33" s="9">
+      <c r="J33" s="10">
         <v>2</v>
       </c>
-      <c r="K33" s="9"/>
-    </row>
-    <row r="34" ht="36.75" spans="1:11">
-      <c r="A34" s="2"/>
-      <c r="B34" s="7">
+      <c r="K33" s="10"/>
+    </row>
+    <row r="34" spans="1:11">
+      <c r="A34" s="3"/>
+      <c r="B34" s="8">
         <f>ROW(B34)-ROW($B$2)</f>
         <v>32</v>
       </c>
-      <c r="C34" s="11" t="s">
-        <v>164</v>
+      <c r="C34" s="14" t="s">
+        <v>156</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I34" s="13" t="s">
         <v>81</v>
@@ -3315,776 +3336,780 @@
       </c>
       <c r="K34" s="12"/>
     </row>
-    <row r="35" ht="36.75" spans="1:11">
-      <c r="A35" s="2"/>
-      <c r="B35" s="7">
+    <row r="35" spans="1:11">
+      <c r="A35" s="3"/>
+      <c r="B35" s="8">
         <f>ROW(B35)-ROW($B$2)</f>
         <v>33</v>
       </c>
-      <c r="C35" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="E35" s="10" t="s">
+      <c r="C35" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="F35" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="G35" s="10" t="s">
+      <c r="D35" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="H35" s="9" t="s">
+      <c r="E35" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="I35" s="13" t="s">
+      <c r="F35" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="G35" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="I35" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J35" s="9">
-        <v>2</v>
-      </c>
-      <c r="K35" s="9"/>
-    </row>
-    <row r="36" ht="15.75" spans="1:11">
-      <c r="A36" s="2"/>
-      <c r="B36" s="7">
+      <c r="J35" s="10">
+        <v>1</v>
+      </c>
+      <c r="K35" s="10"/>
+    </row>
+    <row r="36" spans="1:11">
+      <c r="A36" s="3"/>
+      <c r="B36" s="8">
         <f>ROW(B36)-ROW($B$2)</f>
         <v>34</v>
       </c>
-      <c r="C36" s="11" t="s">
-        <v>174</v>
+      <c r="C36" s="14" t="s">
+        <v>177</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>178</v>
+        <v>92</v>
       </c>
       <c r="I36" s="13" t="s">
         <v>81</v>
       </c>
       <c r="J36" s="12">
-        <v>2</v>
-      </c>
-      <c r="K36" s="12"/>
-    </row>
-    <row r="37" ht="15.75" spans="1:11">
-      <c r="A37" s="2"/>
-      <c r="B37" s="7">
+        <v>1</v>
+      </c>
+      <c r="K36" s="21" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11">
+      <c r="A37" s="3"/>
+      <c r="B37" s="8">
         <f>ROW(B37)-ROW($B$2)</f>
         <v>35</v>
       </c>
-      <c r="C37" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="D37" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="E37" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="F37" s="9" t="s">
+      <c r="C37" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="G37" s="10" t="s">
+      <c r="D37" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="H37" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="I37" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="J37" s="9">
+      <c r="E37" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="G37" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I37" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="J37" s="10">
         <v>1</v>
       </c>
-      <c r="K37" s="9"/>
-    </row>
-    <row r="38" ht="15.75" spans="1:11">
-      <c r="A38" s="2"/>
-      <c r="B38" s="7">
+      <c r="K37" s="10"/>
+    </row>
+    <row r="38" ht="24.75" spans="1:11">
+      <c r="A38" s="3"/>
+      <c r="B38" s="8">
         <f>ROW(B38)-ROW($B$2)</f>
         <v>36</v>
       </c>
-      <c r="C38" s="11" t="s">
-        <v>184</v>
+      <c r="C38" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D38" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="F38" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="E38" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>187</v>
-      </c>
       <c r="G38" s="13" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="H38" s="12" t="s">
         <v>33</v>
       </c>
       <c r="I38" s="13" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="J38" s="12">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="K38" s="12"/>
     </row>
-    <row r="39" ht="24.75" spans="1:11">
-      <c r="A39" s="2"/>
-      <c r="B39" s="7">
+    <row r="39" ht="15.75" spans="1:11">
+      <c r="A39" s="3"/>
+      <c r="B39" s="8">
         <f>ROW(B39)-ROW($B$2)</f>
         <v>37</v>
       </c>
-      <c r="C39" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="D39" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="E39" s="10" t="s">
+      <c r="C39" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="D39" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="F39" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G39" s="10" t="s">
+      <c r="E39" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="H39" s="9" t="s">
+      <c r="F39" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="G39" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="H39" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I39" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="J39" s="9">
-        <v>16</v>
-      </c>
-      <c r="K39" s="9"/>
+      <c r="I39" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="J39" s="10">
+        <v>1</v>
+      </c>
+      <c r="K39" s="10"/>
     </row>
     <row r="40" ht="15.75" spans="1:11">
-      <c r="A40" s="2"/>
-      <c r="B40" s="7">
+      <c r="A40" s="3"/>
+      <c r="B40" s="8">
         <f>ROW(B40)-ROW($B$2)</f>
         <v>38</v>
       </c>
-      <c r="C40" s="8" t="s">
-        <v>190</v>
+      <c r="C40" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="G40" s="13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H40" s="12" t="s">
         <v>33</v>
       </c>
       <c r="I40" s="13" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J40" s="12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K40" s="12"/>
     </row>
-    <row r="41" ht="15.75" spans="1:11">
-      <c r="A41" s="2"/>
-      <c r="B41" s="7">
+    <row r="41" ht="24.75" spans="1:11">
+      <c r="A41" s="3"/>
+      <c r="B41" s="8">
         <f>ROW(B41)-ROW($B$2)</f>
         <v>39</v>
       </c>
-      <c r="C41" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="E41" s="10" t="s">
+      <c r="C41" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D41" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="F41" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G41" s="10" t="s">
+      <c r="E41" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="H41" s="9" t="s">
+      <c r="F41" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="G41" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="H41" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I41" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="J41" s="9">
-        <v>3</v>
-      </c>
-      <c r="K41" s="9"/>
-    </row>
-    <row r="42" ht="24.75" spans="1:11">
-      <c r="A42" s="2"/>
-      <c r="B42" s="7">
+      <c r="I41" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="J41" s="10">
+        <v>13</v>
+      </c>
+      <c r="K41" s="22" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
+      <c r="A42" s="3"/>
+      <c r="B42" s="8">
         <f>ROW(B42)-ROW($B$2)</f>
         <v>40</v>
       </c>
-      <c r="C42" s="8" t="s">
-        <v>190</v>
+      <c r="C42" s="14" t="s">
+        <v>206</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F42" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G42" s="13" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="H42" s="12" t="s">
         <v>33</v>
       </c>
       <c r="I42" s="13" t="s">
-        <v>207</v>
+        <v>151</v>
       </c>
       <c r="J42" s="12">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K42" s="12"/>
     </row>
-    <row r="43" ht="15.75" spans="1:11">
-      <c r="A43" s="2"/>
-      <c r="B43" s="7">
+    <row r="43" spans="1:11">
+      <c r="A43" s="3"/>
+      <c r="B43" s="8">
         <f>ROW(B43)-ROW($B$2)</f>
         <v>41</v>
       </c>
-      <c r="C43" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>208</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="F43" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G43" s="10" t="s">
+      <c r="C43" s="9"/>
+      <c r="D43" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="H43" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="I43" s="10" t="s">
+      <c r="E43" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="J43" s="9">
-        <v>4</v>
-      </c>
-      <c r="K43" s="9"/>
-    </row>
-    <row r="44" ht="36.75" spans="1:11">
-      <c r="A44" s="2"/>
-      <c r="B44" s="7">
+      <c r="F43" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="G43" s="11" t="s">
+        <v>212</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="I43" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="J43" s="10">
+        <v>6</v>
+      </c>
+      <c r="K43" s="10"/>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="A44" s="3"/>
+      <c r="B44" s="8">
         <f>ROW(B44)-ROW($B$2)</f>
         <v>42</v>
       </c>
-      <c r="C44" s="8" t="s">
-        <v>190</v>
+      <c r="C44" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="F44" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G44" s="13" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>215</v>
+        <v>33</v>
       </c>
       <c r="I44" s="13" t="s">
-        <v>216</v>
+        <v>151</v>
       </c>
       <c r="J44" s="12">
-        <v>2</v>
-      </c>
-      <c r="K44" s="12"/>
-    </row>
-    <row r="45" spans="1:11">
-      <c r="A45" s="2"/>
-      <c r="B45" s="7">
+        <v>3</v>
+      </c>
+      <c r="K44" s="21" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="45" ht="15.75" spans="1:11">
+      <c r="A45" s="3"/>
+      <c r="B45" s="8">
         <f>ROW(B45)-ROW($B$2)</f>
         <v>43</v>
       </c>
-      <c r="C45" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="D45" s="9" t="s">
+      <c r="C45" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="E45" s="11" t="s">
         <v>217</v>
       </c>
-      <c r="E45" s="10" t="s">
+      <c r="F45" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="G45" s="11" t="s">
         <v>218</v>
       </c>
-      <c r="F45" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G45" s="10" t="s">
+      <c r="H45" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I45" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="H45" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="I45" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="J45" s="9">
+      <c r="J45" s="10">
         <v>4</v>
       </c>
-      <c r="K45" s="9"/>
-    </row>
-    <row r="46" spans="1:11">
-      <c r="A46" s="2"/>
-      <c r="B46" s="7">
+      <c r="K45" s="10"/>
+    </row>
+    <row r="46" ht="36.75" spans="1:11">
+      <c r="A46" s="3"/>
+      <c r="B46" s="8">
         <f>ROW(B46)-ROW($B$2)</f>
         <v>44</v>
       </c>
-      <c r="C46" s="11" t="s">
-        <v>190</v>
+      <c r="C46" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D46" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="E46" s="13" t="s">
+        <v>221</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="G46" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="E46" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="F46" s="12" t="s">
-        <v>187</v>
-      </c>
-      <c r="G46" s="13" t="s">
-        <v>210</v>
-      </c>
       <c r="H46" s="12" t="s">
-        <v>33</v>
+        <v>223</v>
       </c>
       <c r="I46" s="13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J46" s="12">
         <v>2</v>
       </c>
-      <c r="K46" s="18" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11">
-      <c r="A47" s="2"/>
-      <c r="B47" s="7">
+      <c r="K46" s="12"/>
+    </row>
+    <row r="47" ht="15.75" spans="1:11">
+      <c r="A47" s="3"/>
+      <c r="B47" s="8">
         <f>ROW(B47)-ROW($B$2)</f>
         <v>45</v>
       </c>
-      <c r="C47" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="D47" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="E47" s="10" t="s">
+      <c r="C47" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D47" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="F47" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G47" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="H47" s="9" t="s">
+      <c r="E47" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="G47" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="H47" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I47" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="J47" s="9">
+      <c r="I47" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J47" s="10">
         <v>2</v>
       </c>
-      <c r="K47" s="18" t="s">
-        <v>223</v>
+      <c r="K47" s="22" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="48" spans="1:11">
-      <c r="A48" s="2"/>
-      <c r="B48" s="7">
+      <c r="A48" s="3"/>
+      <c r="B48" s="8">
         <f>ROW(B48)-ROW($B$2)</f>
         <v>46</v>
       </c>
-      <c r="C48" s="11" t="s">
-        <v>190</v>
+      <c r="C48" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D48" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="E48" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="E48" s="13" t="s">
+      <c r="F48" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="G48" s="13" t="s">
         <v>228</v>
-      </c>
-      <c r="F48" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="G48" s="13" t="s">
-        <v>229</v>
       </c>
       <c r="H48" s="12" t="s">
         <v>33</v>
       </c>
       <c r="I48" s="13" t="s">
-        <v>230</v>
+        <v>151</v>
       </c>
       <c r="J48" s="12">
-        <v>1</v>
-      </c>
-      <c r="K48" s="12"/>
+        <v>2</v>
+      </c>
+      <c r="K48" s="22" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="49" ht="15.75" spans="1:11">
-      <c r="A49" s="2"/>
-      <c r="B49" s="7">
+      <c r="A49" s="3"/>
+      <c r="B49" s="8">
         <f>ROW(B49)-ROW($B$2)</f>
         <v>47</v>
       </c>
-      <c r="C49" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="D49" s="9" t="s">
+      <c r="C49" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="E49" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="G49" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="E49" s="10" t="s">
+      <c r="H49" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I49" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="F49" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G49" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="I49" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="J49" s="9">
+      <c r="J49" s="10">
         <v>1</v>
       </c>
-      <c r="K49" s="9"/>
+      <c r="K49" s="10"/>
     </row>
     <row r="50" ht="15.75" spans="1:11">
-      <c r="A50" s="2"/>
-      <c r="B50" s="7">
+      <c r="A50" s="3"/>
+      <c r="B50" s="8">
         <f>ROW(B50)-ROW($B$2)</f>
         <v>48</v>
       </c>
-      <c r="C50" s="11" t="s">
-        <v>190</v>
+      <c r="C50" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>236</v>
+        <v>211</v>
       </c>
       <c r="F50" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G50" s="13" t="s">
-        <v>237</v>
+        <v>212</v>
       </c>
       <c r="H50" s="12" t="s">
-        <v>33</v>
+        <v>213</v>
       </c>
       <c r="I50" s="13" t="s">
-        <v>238</v>
+        <v>151</v>
       </c>
       <c r="J50" s="12">
-        <v>4</v>
-      </c>
-      <c r="K50" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="K50" s="21" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="51" ht="15.75" spans="1:11">
-      <c r="A51" s="2"/>
-      <c r="B51" s="7">
+      <c r="A51" s="3"/>
+      <c r="B51" s="8">
         <f>ROW(B51)-ROW($B$2)</f>
         <v>49</v>
       </c>
-      <c r="C51" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="E51" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G51" s="10" t="s">
-        <v>241</v>
-      </c>
-      <c r="H51" s="9" t="s">
+      <c r="C51" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="E51" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="F51" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="G51" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="H51" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I51" s="10" t="s">
-        <v>242</v>
-      </c>
-      <c r="J51" s="9">
+      <c r="I51" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="J51" s="10">
         <v>1</v>
       </c>
-      <c r="K51" s="9"/>
+      <c r="K51" s="10"/>
     </row>
     <row r="52" ht="15.75" spans="1:11">
-      <c r="A52" s="2"/>
-      <c r="B52" s="7">
+      <c r="A52" s="3"/>
+      <c r="B52" s="8">
         <f>ROW(B52)-ROW($B$2)</f>
         <v>50</v>
       </c>
-      <c r="C52" s="11" t="s">
-        <v>190</v>
+      <c r="C52" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="F52" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G52" s="13" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="H52" s="12" t="s">
         <v>33</v>
       </c>
       <c r="I52" s="13" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="J52" s="12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K52" s="12"/>
     </row>
     <row r="53" ht="15.75" spans="1:11">
-      <c r="A53" s="2"/>
-      <c r="B53" s="7">
+      <c r="A53" s="3"/>
+      <c r="B53" s="8">
         <f>ROW(B53)-ROW($B$2)</f>
         <v>51</v>
       </c>
-      <c r="C53" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="D53" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="E53" s="10" t="s">
-        <v>248</v>
-      </c>
-      <c r="F53" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G53" s="10" t="s">
-        <v>249</v>
-      </c>
-      <c r="H53" s="9" t="s">
+      <c r="C53" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="E53" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="G53" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="H53" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I53" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="J53" s="9">
+      <c r="I53" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="J53" s="10">
         <v>1</v>
       </c>
-      <c r="K53" s="9"/>
+      <c r="K53" s="10"/>
     </row>
     <row r="54" ht="15.75" spans="1:11">
-      <c r="A54" s="2"/>
-      <c r="B54" s="7">
+      <c r="A54" s="3"/>
+      <c r="B54" s="8">
         <f>ROW(B54)-ROW($B$2)</f>
         <v>52</v>
       </c>
-      <c r="C54" s="11" t="s">
-        <v>190</v>
+      <c r="C54" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="F54" s="12" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="G54" s="13" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="H54" s="12" t="s">
         <v>33</v>
       </c>
       <c r="I54" s="13" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="J54" s="12">
         <v>1</v>
       </c>
       <c r="K54" s="12"/>
     </row>
-    <row r="55" spans="1:11">
-      <c r="A55" s="2"/>
-      <c r="B55" s="7">
+    <row r="55" ht="15.75" spans="1:11">
+      <c r="A55" s="3"/>
+      <c r="B55" s="8">
         <f>ROW(B55)-ROW($B$2)</f>
         <v>53</v>
       </c>
-      <c r="C55" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="D55" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="E55" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="F55" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G55" s="10" t="s">
-        <v>257</v>
-      </c>
-      <c r="H55" s="9" t="s">
+      <c r="C55" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="E55" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="G55" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="H55" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I55" s="10" t="s">
-        <v>258</v>
-      </c>
-      <c r="J55" s="9">
-        <v>3</v>
-      </c>
-      <c r="K55" s="9"/>
+      <c r="I55" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="J55" s="10">
+        <v>1</v>
+      </c>
+      <c r="K55" s="10"/>
     </row>
     <row r="56" spans="1:11">
-      <c r="A56" s="2"/>
-      <c r="B56" s="7">
+      <c r="A56" s="3"/>
+      <c r="B56" s="8">
         <f>ROW(B56)-ROW($B$2)</f>
         <v>54</v>
       </c>
-      <c r="C56" s="11" t="s">
-        <v>190</v>
+      <c r="C56" s="14" t="s">
+        <v>206</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>205</v>
+        <v>255</v>
       </c>
       <c r="F56" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G56" s="13" t="s">
-        <v>206</v>
+        <v>256</v>
       </c>
       <c r="H56" s="12" t="s">
         <v>33</v>
       </c>
       <c r="I56" s="13" t="s">
-        <v>223</v>
+        <v>257</v>
       </c>
       <c r="J56" s="12">
-        <v>1</v>
-      </c>
-      <c r="K56" s="18" t="s">
-        <v>223</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="K56" s="12"/>
     </row>
     <row r="57" spans="1:11">
-      <c r="A57" s="2"/>
-      <c r="B57" s="7">
+      <c r="A57" s="3"/>
+      <c r="B57" s="8">
         <f>ROW(B57)-ROW($B$2)</f>
         <v>55</v>
       </c>
-      <c r="C57" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="D57" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="E57" s="10" t="s">
+      <c r="C57" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="E57" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="F57" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="G57" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="F57" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G57" s="10" t="s">
-        <v>257</v>
-      </c>
-      <c r="H57" s="9" t="s">
+      <c r="H57" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I57" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="J57" s="9">
+      <c r="I57" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J57" s="10">
         <v>1</v>
       </c>
-      <c r="K57" s="18" t="s">
-        <v>223</v>
+      <c r="K57" s="22" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="58" ht="24.75" spans="1:11">
-      <c r="A58" s="2"/>
-      <c r="B58" s="7">
+      <c r="A58" s="3"/>
+      <c r="B58" s="8">
         <f>ROW(B58)-ROW($B$2)</f>
         <v>56</v>
       </c>
-      <c r="C58" s="11" t="s">
-        <v>190</v>
+      <c r="C58" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D58" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>260</v>
+      </c>
+      <c r="F58" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="G58" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="E58" s="13" t="s">
+      <c r="H58" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="F58" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="G58" s="13" t="s">
+      <c r="I58" s="13" t="s">
         <v>263</v>
-      </c>
-      <c r="H58" s="12" t="s">
-        <v>264</v>
-      </c>
-      <c r="I58" s="13" t="s">
-        <v>265</v>
       </c>
       <c r="J58" s="12">
         <v>1</v>
@@ -4092,190 +4117,190 @@
       <c r="K58" s="12"/>
     </row>
     <row r="59" ht="24.75" spans="1:11">
-      <c r="A59" s="2"/>
-      <c r="B59" s="7">
+      <c r="A59" s="3"/>
+      <c r="B59" s="8">
         <f>ROW(B59)-ROW($B$2)</f>
         <v>57</v>
       </c>
-      <c r="C59" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="D59" s="9" t="s">
+      <c r="C59" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="E59" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="F59" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="E59" s="10" t="s">
+      <c r="G59" s="11" t="s">
         <v>267</v>
       </c>
-      <c r="F59" s="9" t="s">
+      <c r="H59" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="I59" s="11" t="s">
         <v>268</v>
       </c>
-      <c r="G59" s="10" t="s">
-        <v>269</v>
-      </c>
-      <c r="H59" s="9" t="s">
-        <v>264</v>
-      </c>
-      <c r="I59" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="J59" s="9">
+      <c r="J59" s="10">
         <v>1</v>
       </c>
-      <c r="K59" s="9"/>
+      <c r="K59" s="10"/>
     </row>
     <row r="60" ht="36.75" spans="1:11">
-      <c r="A60" s="2"/>
-      <c r="B60" s="7">
+      <c r="A60" s="3"/>
+      <c r="B60" s="8">
         <f>ROW(B60)-ROW($B$2)</f>
         <v>58</v>
       </c>
-      <c r="C60" s="11" t="s">
-        <v>190</v>
+      <c r="C60" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="D60" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E60" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="F60" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="G60" s="13" t="s">
         <v>271</v>
       </c>
-      <c r="E60" s="13" t="s">
+      <c r="H60" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="I60" s="13" t="s">
         <v>272</v>
-      </c>
-      <c r="F60" s="12" t="s">
-        <v>268</v>
-      </c>
-      <c r="G60" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="H60" s="12" t="s">
-        <v>264</v>
-      </c>
-      <c r="I60" s="13" t="s">
-        <v>274</v>
       </c>
       <c r="J60" s="12">
         <v>1</v>
       </c>
       <c r="K60" s="12"/>
     </row>
-    <row r="61" spans="1:11">
-      <c r="A61" s="2"/>
-      <c r="B61" s="7">
+    <row r="61" ht="15.75" spans="1:11">
+      <c r="A61" s="3"/>
+      <c r="B61" s="8">
         <f>ROW(B61)-ROW($B$2)</f>
         <v>59</v>
       </c>
-      <c r="C61" s="8" t="s">
+      <c r="C61" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="E61" s="11" t="s">
         <v>275</v>
       </c>
-      <c r="D61" s="9" t="s">
+      <c r="F61" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="E61" s="10" t="s">
+      <c r="G61" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="H61" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="F61" s="9" t="s">
-        <v>278</v>
-      </c>
-      <c r="G61" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="H61" s="9" t="s">
-        <v>279</v>
-      </c>
-      <c r="I61" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="J61" s="9">
+      <c r="I61" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J61" s="10">
         <v>1</v>
       </c>
-      <c r="K61" s="19" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11">
-      <c r="A62" s="2"/>
-      <c r="B62" s="7">
+      <c r="K61" s="22" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="62" ht="36.75" spans="1:11">
+      <c r="A62" s="3"/>
+      <c r="B62" s="8">
         <f>ROW(B62)-ROW($B$2)</f>
         <v>60</v>
       </c>
-      <c r="C62" s="11" t="s">
-        <v>275</v>
+      <c r="C62" s="9" t="s">
+        <v>273</v>
       </c>
       <c r="D62" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="E62" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="F62" s="12" t="s">
         <v>280</v>
       </c>
-      <c r="E62" s="13" t="s">
-        <v>277</v>
-      </c>
-      <c r="F62" s="12" t="s">
-        <v>278</v>
-      </c>
       <c r="G62" s="13" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="H62" s="12" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="I62" s="13" t="s">
         <v>81</v>
       </c>
       <c r="J62" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K62" s="12"/>
     </row>
-    <row r="63" ht="36.75" spans="1:11">
-      <c r="A63" s="2"/>
-      <c r="B63" s="7">
+    <row r="63" ht="15.75" spans="1:11">
+      <c r="A63" s="3"/>
+      <c r="B63" s="8">
         <f>ROW(B63)-ROW($B$2)</f>
         <v>61</v>
       </c>
-      <c r="C63" s="11" t="s">
-        <v>275</v>
-      </c>
-      <c r="D63" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="E63" s="10" t="s">
+      <c r="C63" s="9" t="s">
         <v>282</v>
       </c>
-      <c r="F63" s="9" t="s">
+      <c r="D63" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="G63" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="H63" s="9" t="s">
+      <c r="E63" s="11" t="s">
         <v>284</v>
       </c>
-      <c r="I63" s="13" t="s">
+      <c r="F63" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="G63" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="H63" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="I63" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J63" s="9">
+      <c r="J63" s="10">
         <v>1</v>
       </c>
-      <c r="K63" s="9"/>
+      <c r="K63" s="10"/>
     </row>
     <row r="64" ht="15.75" spans="1:11">
-      <c r="A64" s="2"/>
-      <c r="B64" s="7">
+      <c r="A64" s="3"/>
+      <c r="B64" s="8">
         <f>ROW(B64)-ROW($B$2)</f>
         <v>62</v>
       </c>
-      <c r="C64" s="11" t="s">
-        <v>285</v>
+      <c r="C64" s="14" t="s">
+        <v>282</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E64" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="F64" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="G64" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="H64" s="12" t="s">
         <v>287</v>
-      </c>
-      <c r="F64" s="12" t="s">
-        <v>288</v>
-      </c>
-      <c r="G64" s="13" t="s">
-        <v>289</v>
-      </c>
-      <c r="H64" s="12" t="s">
-        <v>290</v>
       </c>
       <c r="I64" s="13" t="s">
         <v>81</v>
@@ -4285,61 +4310,61 @@
       </c>
       <c r="K64" s="12"/>
     </row>
-    <row r="65" ht="15.75" spans="1:11">
-      <c r="A65" s="2"/>
-      <c r="B65" s="7">
+    <row r="65" ht="24.75" spans="1:11">
+      <c r="A65" s="3"/>
+      <c r="B65" s="8">
         <f>ROW(B65)-ROW($B$2)</f>
         <v>63</v>
       </c>
-      <c r="C65" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="D65" s="9" t="s">
+      <c r="C65" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="D65" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="E65" s="10" t="s">
+      <c r="E65" s="11" t="s">
         <v>293</v>
       </c>
-      <c r="F65" s="9" t="s">
+      <c r="F65" s="10" t="s">
         <v>294</v>
       </c>
-      <c r="G65" s="10" t="s">
+      <c r="G65" s="11" t="s">
         <v>295</v>
       </c>
-      <c r="H65" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="I65" s="13" t="s">
+      <c r="H65" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="I65" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J65" s="9">
+      <c r="J65" s="10">
         <v>1</v>
       </c>
-      <c r="K65" s="9"/>
-    </row>
-    <row r="66" ht="24.75" spans="1:11">
-      <c r="A66" s="2"/>
-      <c r="B66" s="7">
+      <c r="K65" s="10"/>
+    </row>
+    <row r="66" ht="15.75" spans="1:11">
+      <c r="A66" s="3"/>
+      <c r="B66" s="8">
         <f>ROW(B66)-ROW($B$2)</f>
         <v>64</v>
       </c>
-      <c r="C66" s="11" t="s">
-        <v>285</v>
+      <c r="C66" s="14" t="s">
+        <v>282</v>
       </c>
       <c r="D66" s="12" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F66" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G66" s="13" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="I66" s="13" t="s">
         <v>81</v>
@@ -4349,108 +4374,108 @@
       </c>
       <c r="K66" s="12"/>
     </row>
-    <row r="67" ht="15.75" spans="1:11">
-      <c r="A67" s="2"/>
-      <c r="B67" s="7">
+    <row r="67" ht="36.75" spans="1:11">
+      <c r="A67" s="3"/>
+      <c r="B67" s="8">
         <f>ROW(B67)-ROW($B$2)</f>
         <v>65</v>
       </c>
-      <c r="C67" s="11" t="s">
-        <v>285</v>
-      </c>
-      <c r="D67" s="9" t="s">
-        <v>301</v>
-      </c>
-      <c r="E67" s="10" t="s">
+      <c r="C67" s="9" t="s">
         <v>302</v>
       </c>
-      <c r="F67" s="9" t="s">
+      <c r="D67" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="G67" s="10" t="s">
+      <c r="E67" s="11" t="s">
         <v>304</v>
       </c>
-      <c r="H67" s="9" t="s">
+      <c r="F67" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="G67" s="11" t="s">
         <v>305</v>
       </c>
-      <c r="I67" s="13" t="s">
+      <c r="H67" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="I67" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J67" s="9">
-        <v>1</v>
-      </c>
-      <c r="K67" s="9"/>
-    </row>
-    <row r="68" ht="36.75" spans="1:11">
-      <c r="A68" s="2"/>
-      <c r="B68" s="7">
+      <c r="J67" s="10">
+        <v>4</v>
+      </c>
+      <c r="K67" s="10"/>
+    </row>
+    <row r="68" ht="24.75" spans="1:11">
+      <c r="A68" s="3"/>
+      <c r="B68" s="8">
         <f>ROW(B68)-ROW($B$2)</f>
         <v>66</v>
       </c>
-      <c r="C68" s="11" t="s">
-        <v>306</v>
+      <c r="C68" s="14" t="s">
+        <v>307</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F68" s="12" t="s">
-        <v>309</v>
+        <v>102</v>
       </c>
       <c r="G68" s="13" t="s">
-        <v>309</v>
-      </c>
-      <c r="H68" s="12" t="s">
         <v>310</v>
       </c>
+      <c r="H68" s="12"/>
       <c r="I68" s="13" t="s">
         <v>81</v>
       </c>
       <c r="J68" s="12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K68" s="12"/>
     </row>
-    <row r="69" ht="24.75" spans="1:11">
-      <c r="A69" s="2"/>
-      <c r="B69" s="7">
+    <row r="69" spans="1:11">
+      <c r="A69" s="3"/>
+      <c r="B69" s="8">
         <f>ROW(B69)-ROW($B$2)</f>
         <v>67</v>
       </c>
-      <c r="C69" s="8" t="s">
+      <c r="C69" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="D69" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="D69" s="9" t="s">
+      <c r="E69" s="11" t="s">
         <v>312</v>
       </c>
-      <c r="E69" s="10" t="s">
+      <c r="F69" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="F69" s="9" t="s">
+      <c r="G69" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="G69" s="10" t="s">
-        <v>314</v>
-      </c>
-      <c r="H69" s="9"/>
-      <c r="I69" s="13" t="s">
+      <c r="H69" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="I69" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J69" s="9">
+      <c r="J69" s="10">
         <v>1</v>
       </c>
-      <c r="K69" s="9"/>
-    </row>
-    <row r="70" ht="15.75" spans="1:11">
-      <c r="A70" s="2"/>
-      <c r="B70" s="7">
+      <c r="K69" s="10"/>
+    </row>
+    <row r="70" spans="1:11">
+      <c r="A70" s="3"/>
+      <c r="B70" s="8">
         <f>ROW(B70)-ROW($B$2)</f>
         <v>68</v>
       </c>
-      <c r="C70" s="11" t="s">
-        <v>285</v>
+      <c r="C70" s="14" t="s">
+        <v>282</v>
       </c>
       <c r="D70" s="12" t="s">
         <v>315</v>
@@ -4465,9 +4490,9 @@
         <v>318</v>
       </c>
       <c r="H70" s="12" t="s">
-        <v>290</v>
-      </c>
-      <c r="I70" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="I70" s="11" t="s">
         <v>81</v>
       </c>
       <c r="J70" s="12">
@@ -4475,63 +4500,63 @@
       </c>
       <c r="K70" s="12"/>
     </row>
-    <row r="71" ht="15.75" spans="1:11">
-      <c r="A71" s="2"/>
-      <c r="B71" s="7">
+    <row r="71" spans="1:11">
+      <c r="A71" s="3"/>
+      <c r="B71" s="8">
         <f>ROW(B71)-ROW($B$2)</f>
         <v>69</v>
       </c>
-      <c r="C71" s="8" t="s">
-        <v>285</v>
-      </c>
-      <c r="D71" s="9" t="s">
+      <c r="C71" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="D71" s="10" t="s">
         <v>319</v>
       </c>
-      <c r="E71" s="10" t="s">
+      <c r="E71" s="11" t="s">
         <v>320</v>
       </c>
-      <c r="F71" s="9" t="s">
+      <c r="F71" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="G71" s="11" t="s">
         <v>321</v>
       </c>
-      <c r="G71" s="10" t="s">
-        <v>322</v>
-      </c>
-      <c r="H71" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="I71" s="13" t="s">
+      <c r="H71" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="I71" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J71" s="9">
+      <c r="J71" s="10">
         <v>1</v>
       </c>
-      <c r="K71" s="9"/>
-    </row>
-    <row r="72" ht="15.75" spans="1:11">
-      <c r="A72" s="2"/>
-      <c r="B72" s="7">
+      <c r="K71" s="10"/>
+    </row>
+    <row r="72" spans="1:11">
+      <c r="A72" s="3"/>
+      <c r="B72" s="8">
         <f>ROW(B72)-ROW($B$2)</f>
         <v>70</v>
       </c>
-      <c r="C72" s="11" t="s">
-        <v>285</v>
+      <c r="C72" s="14" t="s">
+        <v>282</v>
       </c>
       <c r="D72" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="E72" s="13" t="s">
         <v>323</v>
       </c>
-      <c r="E72" s="13" t="s">
+      <c r="F72" s="12" t="s">
         <v>324</v>
-      </c>
-      <c r="F72" s="12" t="s">
-        <v>294</v>
       </c>
       <c r="G72" s="13" t="s">
         <v>325</v>
       </c>
       <c r="H72" s="12" t="s">
-        <v>290</v>
-      </c>
-      <c r="I72" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="I72" s="11" t="s">
         <v>81</v>
       </c>
       <c r="J72" s="12">
@@ -4539,63 +4564,63 @@
       </c>
       <c r="K72" s="12"/>
     </row>
-    <row r="73" ht="15.75" spans="1:11">
-      <c r="A73" s="2"/>
-      <c r="B73" s="7">
+    <row r="73" ht="24.75" spans="1:11">
+      <c r="A73" s="3"/>
+      <c r="B73" s="8">
         <f>ROW(B73)-ROW($B$2)</f>
         <v>71</v>
       </c>
-      <c r="C73" s="8" t="s">
-        <v>285</v>
-      </c>
-      <c r="D73" s="9" t="s">
+      <c r="C73" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="D73" s="10" t="s">
         <v>326</v>
       </c>
-      <c r="E73" s="10" t="s">
+      <c r="E73" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="F73" s="9" t="s">
+      <c r="F73" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="G73" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="H73" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="I73" s="13" t="s">
+      <c r="G73" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="H73" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="I73" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J73" s="9">
+      <c r="J73" s="10">
         <v>1</v>
       </c>
-      <c r="K73" s="9"/>
-    </row>
-    <row r="74" ht="24.75" spans="1:11">
-      <c r="A74" s="2"/>
-      <c r="B74" s="7">
+      <c r="K73" s="10"/>
+    </row>
+    <row r="74" spans="1:11">
+      <c r="A74" s="3"/>
+      <c r="B74" s="8">
         <f>ROW(B74)-ROW($B$2)</f>
         <v>72</v>
       </c>
-      <c r="C74" s="11" t="s">
-        <v>285</v>
+      <c r="C74" s="14" t="s">
+        <v>282</v>
       </c>
       <c r="D74" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="E74" s="13" t="s">
         <v>330</v>
       </c>
-      <c r="E74" s="13" t="s">
+      <c r="F74" s="12" t="s">
         <v>331</v>
-      </c>
-      <c r="F74" s="12" t="s">
-        <v>332</v>
       </c>
       <c r="G74" s="13" t="s">
         <v>332</v>
       </c>
       <c r="H74" s="12" t="s">
-        <v>290</v>
-      </c>
-      <c r="I74" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="I74" s="11" t="s">
         <v>81</v>
       </c>
       <c r="J74" s="12">
@@ -4603,133 +4628,101 @@
       </c>
       <c r="K74" s="12"/>
     </row>
-    <row r="75" ht="15.75" spans="1:11">
-      <c r="A75" s="2"/>
-      <c r="B75" s="7">
+    <row r="75" spans="1:11">
+      <c r="A75" s="3"/>
+      <c r="B75" s="8">
         <f>ROW(B75)-ROW($B$2)</f>
         <v>73</v>
       </c>
-      <c r="C75" s="8" t="s">
-        <v>285</v>
-      </c>
-      <c r="D75" s="9" t="s">
+      <c r="C75" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="D75" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="E75" s="10" t="s">
+      <c r="E75" s="11" t="s">
         <v>334</v>
       </c>
-      <c r="F75" s="9" t="s">
+      <c r="F75" s="10" t="s">
         <v>335</v>
       </c>
-      <c r="G75" s="10" t="s">
+      <c r="G75" s="11" t="s">
         <v>336</v>
       </c>
-      <c r="H75" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="I75" s="13" t="s">
+      <c r="H75" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="I75" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J75" s="9">
+      <c r="J75" s="10">
         <v>1</v>
       </c>
-      <c r="K75" s="9"/>
-    </row>
-    <row r="76" ht="15.75" spans="1:11">
-      <c r="A76" s="2"/>
-      <c r="B76" s="7">
+      <c r="K75" s="10"/>
+    </row>
+    <row r="76" ht="36.75" spans="1:11">
+      <c r="A76" s="3"/>
+      <c r="B76" s="8">
         <f>ROW(B76)-ROW($B$2)</f>
         <v>74</v>
       </c>
-      <c r="C76" s="11" t="s">
-        <v>285</v>
+      <c r="C76" s="14" t="s">
+        <v>338</v>
       </c>
       <c r="D76" s="12" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F76" s="12" t="s">
-        <v>339</v>
+        <v>102</v>
       </c>
       <c r="G76" s="13" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H76" s="12" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="I76" s="13" t="s">
-        <v>81</v>
+        <v>343</v>
       </c>
       <c r="J76" s="12">
         <v>1</v>
       </c>
       <c r="K76" s="12"/>
     </row>
-    <row r="77" ht="36.75" spans="1:11">
-      <c r="A77" s="2"/>
-      <c r="B77" s="7">
+    <row r="77" ht="24.75" spans="1:11">
+      <c r="A77" s="3"/>
+      <c r="B77" s="8">
         <f>ROW(B77)-ROW($B$2)</f>
         <v>75</v>
       </c>
-      <c r="C77" s="8" t="s">
-        <v>342</v>
-      </c>
-      <c r="D77" s="9" t="s">
-        <v>343</v>
-      </c>
-      <c r="E77" s="10" t="s">
+      <c r="C77" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="D77" s="10" t="s">
         <v>344</v>
       </c>
-      <c r="F77" s="9" t="s">
+      <c r="E77" s="11" t="s">
         <v>345</v>
       </c>
-      <c r="G77" s="10" t="s">
-        <v>345</v>
-      </c>
-      <c r="H77" s="9" t="s">
+      <c r="F77" s="10" t="s">
         <v>346</v>
       </c>
-      <c r="I77" s="10" t="s">
+      <c r="G77" s="11" t="s">
         <v>347</v>
       </c>
-      <c r="J77" s="9">
+      <c r="H77" s="10" t="s">
+        <v>348</v>
+      </c>
+      <c r="I77" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="J77" s="10">
         <v>1</v>
       </c>
-      <c r="K77" s="9"/>
-    </row>
-    <row r="78" ht="24.75" spans="1:11">
-      <c r="A78" s="2"/>
-      <c r="B78" s="7">
-        <f>ROW(B78)-ROW($B$2)</f>
-        <v>76</v>
-      </c>
-      <c r="C78" s="11" t="s">
-        <v>342</v>
-      </c>
-      <c r="D78" s="12" t="s">
-        <v>348</v>
-      </c>
-      <c r="E78" s="13" t="s">
-        <v>349</v>
-      </c>
-      <c r="F78" s="12" t="s">
-        <v>350</v>
-      </c>
-      <c r="G78" s="13" t="s">
-        <v>351</v>
-      </c>
-      <c r="H78" s="12" t="s">
-        <v>352</v>
-      </c>
-      <c r="I78" s="13" t="s">
-        <v>353</v>
-      </c>
-      <c r="J78" s="12">
-        <v>1</v>
-      </c>
-      <c r="K78" s="12"/>
+      <c r="K77" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>